<commit_message>
#59 common/npc 스크립트 제거
</commit_message>
<xml_diff>
--- a/resources/table/npc.xlsx
+++ b/resources/table/npc.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\fb\resources\table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F658EDF-46DA-4D37-A63B-56604A0F6685}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34815169-6DBF-44AF-88CB-63887FF57B1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{2AD1A0EA-2C47-4BED-8190-24EDA4F164BF}"/>
+    <workbookView xWindow="32220" yWindow="3420" windowWidth="21600" windowHeight="11385" xr2:uid="{2AD1A0EA-2C47-4BED-8190-24EDA4F164BF}"/>
   </bookViews>
   <sheets>
     <sheet name="npc" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
fix: resolve dialog portrait system compilation issues
- Change portrait from unique_ptr to raw pointer for lambda capture compatibility
- Fix shield data type from uint16_t to uint8_t across all systems
- Update Lua script to use portrait instead of preset parameter
- Simplify model structure by removing optional types for weapon/armor/shield
- Fix Lua table access index from 6 to 2 for portrait parameters
- Update serialization to match new data types
</commit_message>
<xml_diff>
--- a/resources/table/npc.xlsx
+++ b/resources/table/npc.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\fb\resources\table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F77AD699-3415-4657-8589-5428B35F9EA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB3CD438-5A5A-4F56-B425-67F974A3A679}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{2AD1A0EA-2C47-4BED-8190-24EDA4F164BF}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{2AD1A0EA-2C47-4BED-8190-24EDA4F164BF}"/>
   </bookViews>
   <sheets>
     <sheet name="npc" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6570" uniqueCount="2296">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6570" uniqueCount="2295">
   <si>
     <t>id</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -6964,10 +6964,6 @@
   </si>
   <si>
     <t>weapon</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>$item?</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -7512,7 +7508,7 @@
         <v>2266</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>2292</v>
+        <v>2291</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
@@ -7544,7 +7540,7 @@
         <v>2271</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>2293</v>
+        <v>2292</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
@@ -13241,10 +13237,10 @@
     </row>
     <row r="253" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A253" s="1" t="s">
+        <v>2289</v>
+      </c>
+      <c r="B253" s="1" t="s">
         <v>2290</v>
-      </c>
-      <c r="B253" s="1" t="s">
-        <v>2291</v>
       </c>
       <c r="C253" s="1" t="s">
         <v>1521</v>
@@ -13293,34 +13289,34 @@
         <v>2272</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>2286</v>
+        <v>2285</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>2288</v>
+        <v>2287</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>2274</v>
       </c>
       <c r="F1" s="2" t="s">
+        <v>2275</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>2276</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>2277</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>2278</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
+        <v>2294</v>
+      </c>
+      <c r="K1" s="2" t="s">
         <v>2279</v>
       </c>
-      <c r="J1" s="2" t="s">
-        <v>2295</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>2280</v>
-      </c>
       <c r="L1" s="2" t="s">
-        <v>2282</v>
+        <v>2281</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.3">
@@ -13331,34 +13327,34 @@
         <v>2273</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>2287</v>
+        <v>2286</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>2289</v>
+        <v>2288</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>2275</v>
+        <v>2286</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>2289</v>
+        <v>2288</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>2275</v>
+        <v>2286</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>2289</v>
+        <v>2288</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>2275</v>
+        <v>2288</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>2289</v>
+        <v>2288</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>2281</v>
+        <v>2280</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>2283</v>
+        <v>2282</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.3">
@@ -13404,7 +13400,7 @@
         <v>1</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>2284</v>
+        <v>2283</v>
       </c>
       <c r="C4" s="2">
         <v>0</v>
@@ -13412,17 +13408,26 @@
       <c r="D4" s="2">
         <v>0</v>
       </c>
+      <c r="E4" s="2">
+        <v>60</v>
+      </c>
       <c r="F4" s="2">
         <v>0</v>
       </c>
+      <c r="G4" s="2">
+        <v>2</v>
+      </c>
       <c r="H4" s="2">
         <v>0</v>
       </c>
+      <c r="I4" s="2">
+        <v>16</v>
+      </c>
       <c r="J4" s="2">
         <v>0</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>2285</v>
+        <v>2284</v>
       </c>
     </row>
   </sheetData>
@@ -24908,10 +24913,10 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B6" s="1" t="s">
-        <v>2290</v>
+        <v>2289</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>2294</v>
+        <v>2293</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>657</v>

</xml_diff>

<commit_message>
refactor: extract portrait system and add preset support
- Extract portrait classes from dialog.h to separate portrait.h file
- Add character_portrait constructor to fix aggregate initialization error
- Update all dialog protocols to use fb::game::portrait namespace
- Add preset field to mob and npc models for character appearance
- Implement preset-based portrait generation in listener
- Add new preset.xlsx table for character appearance presets
- Improve code organization and reduce coupling between dialog and portrait systems
</commit_message>
<xml_diff>
--- a/resources/table/npc.xlsx
+++ b/resources/table/npc.xlsx
@@ -5,20 +5,19 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\fb\resources\table\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\fb\resources\table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65801FBF-F0D5-4381-B150-D84FFCA82D21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7154F340-9D20-41A6-B4A2-11577A461E80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{2AD1A0EA-2C47-4BED-8190-24EDA4F164BF}"/>
+    <workbookView xWindow="38280" yWindow="-135" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{2AD1A0EA-2C47-4BED-8190-24EDA4F164BF}"/>
   </bookViews>
   <sheets>
     <sheet name="npc" sheetId="1" r:id="rId1"/>
-    <sheet name="preset" sheetId="7" r:id="rId2"/>
-    <sheet name="sell" sheetId="3" r:id="rId3"/>
-    <sheet name="buy" sheetId="4" r:id="rId4"/>
-    <sheet name="npc_spawn" sheetId="5" r:id="rId5"/>
-    <sheet name="soliloquy" sheetId="6" r:id="rId6"/>
+    <sheet name="sell" sheetId="3" r:id="rId2"/>
+    <sheet name="buy" sheetId="4" r:id="rId3"/>
+    <sheet name="npc_spawn" sheetId="5" r:id="rId4"/>
+    <sheet name="soliloquy" sheetId="6" r:id="rId5"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -30,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6609" uniqueCount="2310">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6565" uniqueCount="2288">
   <si>
     <t>id</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -6955,74 +6954,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>sex</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>SEX</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>weapon</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>weapon_color</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>armor</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>armor_color</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>shield</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>disguise</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>uint16?</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>state</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>STATE</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>MAN</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>NORMAL</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>hair</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>uint16</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>hair_color</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>uint8</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>261</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -7036,26 +6967,6 @@
   </si>
   <si>
     <t>10, 10</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>shield_color</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>uint8?</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>WOMAN</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>GHOST</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>RIDING</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -7197,7 +7108,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="표준" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -7213,7 +7124,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 테마">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
     <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
@@ -7563,7 +7474,7 @@
         <v>2266</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>2290</v>
+        <v>2273</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
@@ -7595,7 +7506,7 @@
         <v>2271</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>2291</v>
+        <v>2274</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
@@ -13292,10 +13203,10 @@
     </row>
     <row r="253" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A253" s="1" t="s">
-        <v>2289</v>
+        <v>2272</v>
       </c>
       <c r="B253" s="1" t="s">
-        <v>2301</v>
+        <v>2279</v>
       </c>
       <c r="C253" s="1" t="s">
         <v>1521</v>
@@ -13318,10 +13229,10 @@
     </row>
     <row r="254" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A254" s="1" t="s">
-        <v>2298</v>
+        <v>2276</v>
       </c>
       <c r="B254" s="1" t="s">
-        <v>2302</v>
+        <v>2280</v>
       </c>
       <c r="C254" s="1" t="s">
         <v>1521</v>
@@ -13344,10 +13255,10 @@
     </row>
     <row r="255" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A255" s="1" t="s">
-        <v>2299</v>
+        <v>2277</v>
       </c>
       <c r="B255" s="1" t="s">
-        <v>2303</v>
+        <v>2281</v>
       </c>
       <c r="C255" s="1" t="s">
         <v>1521</v>
@@ -13370,10 +13281,10 @@
     </row>
     <row r="256" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A256" s="1" t="s">
-        <v>2300</v>
+        <v>2278</v>
       </c>
       <c r="B256" s="1" t="s">
-        <v>2304</v>
+        <v>2282</v>
       </c>
       <c r="C256" s="1" t="s">
         <v>1521</v>
@@ -13405,258 +13316,6 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{72547E2E-7C01-450E-BFAA-AA26DEFD419B}">
-  <dimension ref="A1:L7"/>
-  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="9" width="9" style="2"/>
-    <col min="10" max="10" width="10.375" style="2" bestFit="1" customWidth="1"/>
-    <col min="11" max="16384" width="9" style="2"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>2272</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2285</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>2287</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>2274</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>2275</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>2276</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>2277</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>2278</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>2293</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>2279</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>2281</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>2273</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>2286</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>2288</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>2280</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>2294</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>2280</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>2294</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>2294</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>2294</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>2280</v>
-      </c>
-      <c r="L2" s="2" t="s">
-        <v>2282</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="K3" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="L3" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A4" s="2">
-        <v>1</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>2283</v>
-      </c>
-      <c r="C4" s="2">
-        <v>0</v>
-      </c>
-      <c r="D4" s="2">
-        <v>0</v>
-      </c>
-      <c r="E4" s="2">
-        <v>60</v>
-      </c>
-      <c r="F4" s="2">
-        <v>0</v>
-      </c>
-      <c r="G4" s="2">
-        <v>2</v>
-      </c>
-      <c r="H4" s="2">
-        <v>0</v>
-      </c>
-      <c r="I4" s="2">
-        <v>16</v>
-      </c>
-      <c r="J4" s="2">
-        <v>0</v>
-      </c>
-      <c r="L4" s="2" t="s">
-        <v>2284</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A5" s="2">
-        <v>2</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>2295</v>
-      </c>
-      <c r="C5" s="2">
-        <v>0</v>
-      </c>
-      <c r="D5" s="2">
-        <v>0</v>
-      </c>
-      <c r="E5" s="2">
-        <v>60</v>
-      </c>
-      <c r="F5" s="2">
-        <v>0</v>
-      </c>
-      <c r="I5" s="2">
-        <v>16</v>
-      </c>
-      <c r="J5" s="2">
-        <v>0</v>
-      </c>
-      <c r="L5" s="2" t="s">
-        <v>2284</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A6" s="2">
-        <v>3</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>2283</v>
-      </c>
-      <c r="C6" s="2">
-        <v>0</v>
-      </c>
-      <c r="D6" s="2">
-        <v>0</v>
-      </c>
-      <c r="E6" s="2">
-        <v>60</v>
-      </c>
-      <c r="F6" s="2">
-        <v>0</v>
-      </c>
-      <c r="I6" s="2">
-        <v>16</v>
-      </c>
-      <c r="J6" s="2">
-        <v>0</v>
-      </c>
-      <c r="L6" s="2" t="s">
-        <v>2296</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A7" s="2">
-        <v>4</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>2295</v>
-      </c>
-      <c r="C7" s="2">
-        <v>0</v>
-      </c>
-      <c r="D7" s="2">
-        <v>0</v>
-      </c>
-      <c r="E7" s="2">
-        <v>60</v>
-      </c>
-      <c r="F7" s="2">
-        <v>0</v>
-      </c>
-      <c r="I7" s="2">
-        <v>16</v>
-      </c>
-      <c r="J7" s="2">
-        <v>0</v>
-      </c>
-      <c r="L7" s="2" t="s">
-        <v>2297</v>
-      </c>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{467D91EC-BF40-4F9B-8B8D-6019747193CB}">
   <dimension ref="A1:E756"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
@@ -19231,7 +18890,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22443152-8BD8-489A-B59C-AD30C7EE0DA5}">
   <dimension ref="A1:D790"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
@@ -25063,7 +24722,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3A8B4EC-A9F0-4F37-A700-83BC81A3F915}">
   <dimension ref="A1:D1474"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
@@ -25133,10 +24792,10 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B6" s="1" t="s">
-        <v>2289</v>
+        <v>2272</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>2292</v>
+        <v>2275</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>657</v>
@@ -25144,35 +24803,35 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B7" s="1" t="s">
-        <v>2298</v>
+        <v>2276</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>2305</v>
+        <v>2283</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>2307</v>
+        <v>2285</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B8" s="1" t="s">
-        <v>2299</v>
+        <v>2277</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>2306</v>
+        <v>2284</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>2308</v>
+        <v>2286</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B9" s="1" t="s">
-        <v>2300</v>
+        <v>2278</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>1274</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>2309</v>
+        <v>2287</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
@@ -38141,7 +37800,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{52B925D1-5541-4FEF-A6C8-C42626081064}">
   <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>

</xml_diff>

<commit_message>
script: NPC script implementation and marriage support
- Add and update NPC Lua scripts (wedding officiant, map NPCs, various dialogs)
- Add map scripts and expand interaction.lua and npc.lua
- Add marriage feature: protocol, builtin/character, HTTP model and repository, DB schema
- Update character/server builtins, items, login handler; bot and spell script tweaks
</commit_message>
<xml_diff>
--- a/resources/table/npc.xlsx
+++ b/resources/table/npc.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\fb\resources\table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44090542-2495-48C9-AA48-A33D13FBA94F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68EDC6C7-D805-49B4-9515-EC964468CA41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="npc" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8831" uniqueCount="2264">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7063" uniqueCount="2271">
   <si>
     <t>map</t>
   </si>
@@ -6790,42 +6790,78 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>scripts/npc/원주민장로.lua</t>
-  </si>
-  <si>
-    <t>scripts/npc/찬찬.lua</t>
-  </si>
-  <si>
-    <t>scripts/npc/폭염도미용사.lua</t>
-  </si>
-  <si>
-    <t>scripts/npc/폭염왕장식품.lua</t>
-  </si>
-  <si>
-    <t>scripts/npc/화사화사.lua</t>
-  </si>
-  <si>
-    <t>scripts/npc/화화.lua</t>
-  </si>
-  <si>
-    <t>scripts/npc/환상의섬무당.lua</t>
-  </si>
-  <si>
-    <t>scripts/npc/환상의섬갑옷상.lua</t>
-  </si>
-  <si>
-    <t>scripts/npc/돌순이.lua</t>
-  </si>
-  <si>
-    <t>scripts/npc/돌돌이.lua</t>
-  </si>
-  <si>
     <t>도주영</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>scripts/npc/도주영.lua</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>265</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>266</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>길림미로보초</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>길림동굴보초</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>10</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>scripts/npc/길림미로보초.lua</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>scripts/npc/길림동굴보초.lua</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>NPC_265</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>NPC_266</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>267</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>서쪽태극문보초</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>268</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>동쪽태극문보초</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>scripts/npc/서쪽태극문보초.lua</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>scripts/npc/동쪽태극문보초.lua</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>NPC_267</t>
+  </si>
+  <si>
+    <t>NPC_268</t>
   </si>
 </sst>
 </file>
@@ -7232,7 +7268,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J256"/>
+  <dimension ref="A1:J260"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11" style="1" bestFit="1" customWidth="1"/>
@@ -9709,7 +9745,7 @@
         <v>1292</v>
       </c>
       <c r="B107" s="1" t="s">
-        <v>2262</v>
+        <v>2252</v>
       </c>
       <c r="C107" s="1" t="s">
         <v>1293</v>
@@ -9718,7 +9754,7 @@
         <v>10</v>
       </c>
       <c r="E107" s="1" t="s">
-        <v>2263</v>
+        <v>2253</v>
       </c>
       <c r="F107" s="1" t="s">
         <v>1294</v>
@@ -13257,6 +13293,98 @@
       </c>
       <c r="J256" s="1" t="s">
         <v>33</v>
+      </c>
+    </row>
+    <row r="257" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A257" s="1" t="s">
+        <v>2254</v>
+      </c>
+      <c r="B257" s="1" t="s">
+        <v>2256</v>
+      </c>
+      <c r="C257" s="1" t="s">
+        <v>1634</v>
+      </c>
+      <c r="D257" s="1" t="s">
+        <v>2258</v>
+      </c>
+      <c r="E257" s="1" t="s">
+        <v>2259</v>
+      </c>
+      <c r="F257" s="1" t="s">
+        <v>2261</v>
+      </c>
+      <c r="I257" s="1" t="s">
+        <v>949</v>
+      </c>
+    </row>
+    <row r="258" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A258" s="1" t="s">
+        <v>2255</v>
+      </c>
+      <c r="B258" s="1" t="s">
+        <v>2257</v>
+      </c>
+      <c r="C258" s="1" t="s">
+        <v>1634</v>
+      </c>
+      <c r="D258" s="1" t="s">
+        <v>2258</v>
+      </c>
+      <c r="E258" s="1" t="s">
+        <v>2260</v>
+      </c>
+      <c r="F258" s="1" t="s">
+        <v>2262</v>
+      </c>
+      <c r="I258" s="1" t="s">
+        <v>949</v>
+      </c>
+    </row>
+    <row r="259" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A259" s="1" t="s">
+        <v>2263</v>
+      </c>
+      <c r="B259" s="1" t="s">
+        <v>2264</v>
+      </c>
+      <c r="C259" s="1" t="s">
+        <v>1634</v>
+      </c>
+      <c r="D259" s="1" t="s">
+        <v>2258</v>
+      </c>
+      <c r="E259" s="1" t="s">
+        <v>2267</v>
+      </c>
+      <c r="F259" s="1" t="s">
+        <v>2269</v>
+      </c>
+      <c r="I259" s="1" t="s">
+        <v>949</v>
+      </c>
+    </row>
+    <row r="260" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A260" s="1" t="s">
+        <v>2265</v>
+      </c>
+      <c r="B260" s="1" t="s">
+        <v>2266</v>
+      </c>
+      <c r="C260" s="1" t="s">
+        <v>1634</v>
+      </c>
+      <c r="D260" s="1" t="s">
+        <v>2258</v>
+      </c>
+      <c r="E260" s="1" t="s">
+        <v>2268</v>
+      </c>
+      <c r="F260" s="1" t="s">
+        <v>2270</v>
+      </c>
+      <c r="I260" s="1" t="s">
+        <v>949</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: integration test bug fixes
- Fix async_generator to yield only on co_yield, not co_await task
- Fix thread awaitable callback and result propagation
- Fix Lua error message capture before stack pop
- Remove unused character:spell Lua binding
- Add item-exclude helpers for spell target selection
- Fix spell scripts and 출두 script path
- Update bot integration test hooks and clan dialog assertions
- Improve bot equipment info display
- Regenerate model data and npc table
</commit_message>
<xml_diff>
--- a/resources/table/npc.xlsx
+++ b/resources/table/npc.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\fb\resources\table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B66B700D-D86F-4031-BE3D-FB9C8E7AE991}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB7D9ACF-D0E2-414B-8EFF-081CAFE0C8DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="npc" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9256" uniqueCount="3347">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9256" uniqueCount="3349">
   <si>
     <t>map</t>
   </si>
@@ -10068,6 +10068,28 @@
   </si>
   <si>
     <t>scripts/npc/흑령굴도우미.lua</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2
+3
+4
+5
+6
+7
+8
+9</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>11
+12
+13
+14
+15
+16
+17
+18</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -11015,7 +11037,7 @@
         <v>1183</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>1173</v>
+        <v>3347</v>
       </c>
       <c r="H19" s="3">
         <v>10</v>
@@ -11045,7 +11067,7 @@
         <v>1183</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>1173</v>
+        <v>3347</v>
       </c>
       <c r="H20" s="3">
         <v>10</v>
@@ -11075,7 +11097,7 @@
         <v>1187</v>
       </c>
       <c r="G21" s="5" t="s">
-        <v>30</v>
+        <v>3348</v>
       </c>
       <c r="H21" s="3">
         <v>19</v>
@@ -11105,7 +11127,7 @@
         <v>1189</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>30</v>
+        <v>3348</v>
       </c>
       <c r="H22" s="3">
         <v>19</v>

</xml_diff>

<commit_message>
data: refresh item and npc tables
- Update item.xlsx and npc.xlsx
- Bump generated model timestamps
</commit_message>
<xml_diff>
--- a/resources/table/npc.xlsx
+++ b/resources/table/npc.xlsx
@@ -70139,15 +70139,15 @@
     </row>
     <row r="2044">
       <c r="A2044" s="9" t="n"/>
-      <c r="B2044" t="n">
+      <c r="B2044" s="0" t="n">
         <v>545</v>
       </c>
-      <c r="C2044" t="inlineStr">
+      <c r="C2044" s="0" t="inlineStr">
         <is>
           <t>10, 6</t>
         </is>
       </c>
-      <c r="D2044" t="inlineStr">
+      <c r="D2044" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
@@ -70192,15 +70192,15 @@
     </row>
     <row r="2048">
       <c r="A2048" s="9" t="n"/>
-      <c r="B2048" t="n">
+      <c r="B2048" s="0" t="n">
         <v>444</v>
       </c>
-      <c r="C2048" t="inlineStr">
+      <c r="C2048" s="0" t="inlineStr">
         <is>
           <t>4, 38</t>
         </is>
       </c>
-      <c r="D2048" t="inlineStr">
+      <c r="D2048" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
@@ -70455,15 +70455,15 @@
     </row>
     <row r="2072">
       <c r="A2072" s="9" t="n"/>
-      <c r="B2072" t="n">
+      <c r="B2072" s="0" t="n">
         <v>609</v>
       </c>
-      <c r="C2072" t="inlineStr">
+      <c r="C2072" s="0" t="inlineStr">
         <is>
           <t>14, 14</t>
         </is>
       </c>
-      <c r="D2072" t="inlineStr">
+      <c r="D2072" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
@@ -70479,15 +70479,15 @@
     </row>
     <row r="2074">
       <c r="A2074" s="9" t="n"/>
-      <c r="B2074" t="n">
+      <c r="B2074" s="0" t="n">
         <v>610</v>
       </c>
-      <c r="C2074" t="inlineStr">
+      <c r="C2074" s="0" t="inlineStr">
         <is>
           <t>6, 7</t>
         </is>
       </c>
-      <c r="D2074" t="inlineStr">
+      <c r="D2074" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
@@ -70503,15 +70503,15 @@
     </row>
     <row r="2076">
       <c r="A2076" s="9" t="n"/>
-      <c r="B2076" t="n">
+      <c r="B2076" s="0" t="n">
         <v>612</v>
       </c>
-      <c r="C2076" t="inlineStr">
+      <c r="C2076" s="0" t="inlineStr">
         <is>
           <t>5, 7</t>
         </is>
       </c>
-      <c r="D2076" t="inlineStr">
+      <c r="D2076" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
@@ -70527,15 +70527,15 @@
     </row>
     <row r="2078">
       <c r="A2078" s="9" t="n"/>
-      <c r="B2078" t="n">
+      <c r="B2078" s="0" t="n">
         <v>613</v>
       </c>
-      <c r="C2078" t="inlineStr">
+      <c r="C2078" s="0" t="inlineStr">
         <is>
           <t>6, 5</t>
         </is>
       </c>
-      <c r="D2078" t="inlineStr">
+      <c r="D2078" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
@@ -70551,15 +70551,15 @@
     </row>
     <row r="2080">
       <c r="A2080" s="9" t="n"/>
-      <c r="B2080" t="n">
+      <c r="B2080" s="0" t="n">
         <v>614</v>
       </c>
-      <c r="C2080" t="inlineStr">
+      <c r="C2080" s="0" t="inlineStr">
         <is>
           <t>10, 2</t>
         </is>
       </c>
-      <c r="D2080" t="inlineStr">
+      <c r="D2080" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
@@ -70575,15 +70575,15 @@
     </row>
     <row r="2082">
       <c r="A2082" s="9" t="n"/>
-      <c r="B2082" t="n">
+      <c r="B2082" s="0" t="n">
         <v>615</v>
       </c>
-      <c r="C2082" t="inlineStr">
+      <c r="C2082" s="0" t="inlineStr">
         <is>
           <t>5, 5</t>
         </is>
       </c>
-      <c r="D2082" t="inlineStr">
+      <c r="D2082" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
@@ -70599,15 +70599,15 @@
     </row>
     <row r="2084">
       <c r="A2084" s="9" t="n"/>
-      <c r="B2084" t="n">
+      <c r="B2084" s="0" t="n">
         <v>616</v>
       </c>
-      <c r="C2084" t="inlineStr">
+      <c r="C2084" s="0" t="inlineStr">
         <is>
           <t>6, 5</t>
         </is>
       </c>
-      <c r="D2084" t="inlineStr">
+      <c r="D2084" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
@@ -70623,15 +70623,15 @@
     </row>
     <row r="2086">
       <c r="A2086" s="9" t="n"/>
-      <c r="B2086" t="n">
+      <c r="B2086" s="0" t="n">
         <v>617</v>
       </c>
-      <c r="C2086" t="inlineStr">
+      <c r="C2086" s="0" t="inlineStr">
         <is>
           <t>6, 6</t>
         </is>
       </c>
-      <c r="D2086" t="inlineStr">
+      <c r="D2086" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
@@ -70647,15 +70647,15 @@
     </row>
     <row r="2088">
       <c r="A2088" s="9" t="n"/>
-      <c r="B2088" t="n">
+      <c r="B2088" s="0" t="n">
         <v>618</v>
       </c>
-      <c r="C2088" t="inlineStr">
+      <c r="C2088" s="0" t="inlineStr">
         <is>
           <t>10, 10</t>
         </is>
       </c>
-      <c r="D2088" t="inlineStr">
+      <c r="D2088" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
@@ -70671,15 +70671,15 @@
     </row>
     <row r="2090">
       <c r="A2090" s="9" t="n"/>
-      <c r="B2090" t="n">
+      <c r="B2090" s="0" t="n">
         <v>619</v>
       </c>
-      <c r="C2090" t="inlineStr">
+      <c r="C2090" s="0" t="inlineStr">
         <is>
           <t>7, 7</t>
         </is>
       </c>
-      <c r="D2090" t="inlineStr">
+      <c r="D2090" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
@@ -70695,15 +70695,15 @@
     </row>
     <row r="2092">
       <c r="A2092" s="9" t="n"/>
-      <c r="B2092" t="n">
+      <c r="B2092" s="0" t="n">
         <v>8</v>
       </c>
-      <c r="C2092" t="inlineStr">
+      <c r="C2092" s="0" t="inlineStr">
         <is>
           <t>6, 8</t>
         </is>
       </c>
-      <c r="D2092" t="inlineStr">
+      <c r="D2092" s="0" t="inlineStr">
         <is>
           <t>RIGHT</t>
         </is>
@@ -70719,15 +70719,15 @@
     </row>
     <row r="2094">
       <c r="A2094" s="9" t="n"/>
-      <c r="B2094" t="n">
+      <c r="B2094" s="0" t="n">
         <v>620</v>
       </c>
-      <c r="C2094" t="inlineStr">
+      <c r="C2094" s="0" t="inlineStr">
         <is>
           <t>6, 4</t>
         </is>
       </c>
-      <c r="D2094" t="inlineStr">
+      <c r="D2094" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
@@ -70743,15 +70743,15 @@
     </row>
     <row r="2096">
       <c r="A2096" s="9" t="n"/>
-      <c r="B2096" t="n">
+      <c r="B2096" s="0" t="n">
         <v>621</v>
       </c>
-      <c r="C2096" t="inlineStr">
+      <c r="C2096" s="0" t="inlineStr">
         <is>
           <t>6, 4</t>
         </is>
       </c>
-      <c r="D2096" t="inlineStr">
+      <c r="D2096" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
@@ -70767,15 +70767,15 @@
     </row>
     <row r="2098">
       <c r="A2098" s="9" t="n"/>
-      <c r="B2098" t="n">
+      <c r="B2098" s="0" t="n">
         <v>623</v>
       </c>
-      <c r="C2098" t="inlineStr">
+      <c r="C2098" s="0" t="inlineStr">
         <is>
           <t>6, 4</t>
         </is>
       </c>
-      <c r="D2098" t="inlineStr">
+      <c r="D2098" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
@@ -70791,15 +70791,15 @@
     </row>
     <row r="2100">
       <c r="A2100" s="9" t="n"/>
-      <c r="B2100" t="n">
+      <c r="B2100" s="0" t="n">
         <v>622</v>
       </c>
-      <c r="C2100" t="inlineStr">
+      <c r="C2100" s="0" t="inlineStr">
         <is>
           <t>62, 14</t>
         </is>
       </c>
-      <c r="D2100" t="inlineStr">
+      <c r="D2100" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
@@ -70815,15 +70815,15 @@
     </row>
     <row r="2102">
       <c r="A2102" s="9" t="n"/>
-      <c r="B2102" t="n">
+      <c r="B2102" s="0" t="n">
         <v>624</v>
       </c>
-      <c r="C2102" t="inlineStr">
+      <c r="C2102" s="0" t="inlineStr">
         <is>
           <t>4, 4</t>
         </is>
       </c>
-      <c r="D2102" t="inlineStr">
+      <c r="D2102" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
@@ -70839,15 +70839,15 @@
     </row>
     <row r="2104">
       <c r="A2104" s="9" t="n"/>
-      <c r="B2104" t="n">
+      <c r="B2104" s="0" t="n">
         <v>444</v>
       </c>
-      <c r="C2104" t="inlineStr">
+      <c r="C2104" s="0" t="inlineStr">
         <is>
           <t>3, 5</t>
         </is>
       </c>
-      <c r="D2104" t="inlineStr">
+      <c r="D2104" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
@@ -70887,15 +70887,15 @@
     </row>
     <row r="2108">
       <c r="A2108" s="9" t="n"/>
-      <c r="B2108" t="n">
+      <c r="B2108" s="0" t="n">
         <v>227</v>
       </c>
-      <c r="C2108" t="inlineStr">
+      <c r="C2108" s="0" t="inlineStr">
         <is>
           <t>20, 0</t>
         </is>
       </c>
-      <c r="D2108" t="inlineStr">
+      <c r="D2108" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
@@ -70911,15 +70911,15 @@
     </row>
     <row r="2110">
       <c r="A2110" s="9" t="n"/>
-      <c r="B2110" t="n">
+      <c r="B2110" s="0" t="n">
         <v>227</v>
       </c>
-      <c r="C2110" t="inlineStr">
+      <c r="C2110" s="0" t="inlineStr">
         <is>
           <t>20, 0</t>
         </is>
       </c>
-      <c r="D2110" t="inlineStr">
+      <c r="D2110" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
@@ -70935,15 +70935,15 @@
     </row>
     <row r="2112">
       <c r="A2112" s="9" t="n"/>
-      <c r="B2112" t="n">
+      <c r="B2112" s="0" t="n">
         <v>227</v>
       </c>
-      <c r="C2112" t="inlineStr">
+      <c r="C2112" s="0" t="inlineStr">
         <is>
           <t>20, 0</t>
         </is>
       </c>
-      <c r="D2112" t="inlineStr">
+      <c r="D2112" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
@@ -70959,15 +70959,15 @@
     </row>
     <row r="2114">
       <c r="A2114" s="9" t="n"/>
-      <c r="B2114" t="n">
+      <c r="B2114" s="0" t="n">
         <v>600</v>
       </c>
-      <c r="C2114" t="inlineStr">
+      <c r="C2114" s="0" t="inlineStr">
         <is>
           <t>7, 4</t>
         </is>
       </c>
-      <c r="D2114" t="inlineStr">
+      <c r="D2114" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
@@ -70983,15 +70983,15 @@
     </row>
     <row r="2116">
       <c r="A2116" s="9" t="n"/>
-      <c r="B2116" t="n">
+      <c r="B2116" s="0" t="n">
         <v>458</v>
       </c>
-      <c r="C2116" t="inlineStr">
+      <c r="C2116" s="0" t="inlineStr">
         <is>
           <t>14, 9</t>
         </is>
       </c>
-      <c r="D2116" t="inlineStr">
+      <c r="D2116" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
@@ -71007,15 +71007,15 @@
     </row>
     <row r="2118">
       <c r="A2118" s="9" t="n"/>
-      <c r="B2118" t="n">
+      <c r="B2118" s="0" t="n">
         <v>500</v>
       </c>
-      <c r="C2118" t="inlineStr">
+      <c r="C2118" s="0" t="inlineStr">
         <is>
           <t>13, 10</t>
         </is>
       </c>
-      <c r="D2118" t="inlineStr">
+      <c r="D2118" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
@@ -71031,15 +71031,15 @@
     </row>
     <row r="2120">
       <c r="A2120" s="9" t="n"/>
-      <c r="B2120" t="n">
+      <c r="B2120" s="0" t="n">
         <v>501</v>
       </c>
-      <c r="C2120" t="inlineStr">
+      <c r="C2120" s="0" t="inlineStr">
         <is>
           <t>13, 89</t>
         </is>
       </c>
-      <c r="D2120" t="inlineStr">
+      <c r="D2120" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
@@ -71197,15 +71197,15 @@
     </row>
     <row r="2135">
       <c r="A2135" s="9" t="n"/>
-      <c r="B2135" t="n">
+      <c r="B2135" s="0" t="n">
         <v>28</v>
       </c>
-      <c r="C2135" t="inlineStr">
+      <c r="C2135" s="0" t="inlineStr">
         <is>
           <t>37, 47</t>
         </is>
       </c>
-      <c r="D2135" t="inlineStr">
+      <c r="D2135" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
@@ -71595,15 +71595,15 @@
     </row>
     <row r="2169">
       <c r="A2169" s="9" t="n"/>
-      <c r="B2169" t="n">
+      <c r="B2169" s="0" t="n">
         <v>338</v>
       </c>
-      <c r="C2169" t="inlineStr">
+      <c r="C2169" s="0" t="inlineStr">
         <is>
           <t>25, 25</t>
         </is>
       </c>
-      <c r="D2169" t="inlineStr">
+      <c r="D2169" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
@@ -71627,15 +71627,15 @@
     </row>
     <row r="2171">
       <c r="A2171" s="9" t="n"/>
-      <c r="B2171" t="n">
+      <c r="B2171" s="0" t="n">
         <v>338</v>
       </c>
-      <c r="C2171" t="inlineStr">
+      <c r="C2171" s="0" t="inlineStr">
         <is>
           <t>25, 125</t>
         </is>
       </c>
-      <c r="D2171" t="inlineStr">
+      <c r="D2171" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
@@ -71659,15 +71659,15 @@
     </row>
     <row r="2173">
       <c r="A2173" s="9" t="n"/>
-      <c r="B2173" t="n">
+      <c r="B2173" s="0" t="n">
         <v>338</v>
       </c>
-      <c r="C2173" t="inlineStr">
+      <c r="C2173" s="0" t="inlineStr">
         <is>
           <t>75, 25</t>
         </is>
       </c>
-      <c r="D2173" t="inlineStr">
+      <c r="D2173" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
@@ -71691,15 +71691,15 @@
     </row>
     <row r="2175">
       <c r="A2175" s="9" t="n"/>
-      <c r="B2175" t="n">
+      <c r="B2175" s="0" t="n">
         <v>338</v>
       </c>
-      <c r="C2175" t="inlineStr">
+      <c r="C2175" s="0" t="inlineStr">
         <is>
           <t>75, 125</t>
         </is>
       </c>
-      <c r="D2175" t="inlineStr">
+      <c r="D2175" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
@@ -71723,15 +71723,15 @@
     </row>
     <row r="2177">
       <c r="A2177" s="9" t="n"/>
-      <c r="B2177" t="n">
+      <c r="B2177" s="0" t="n">
         <v>338</v>
       </c>
-      <c r="C2177" t="inlineStr">
+      <c r="C2177" s="0" t="inlineStr">
         <is>
           <t>125, 25</t>
         </is>
       </c>
-      <c r="D2177" t="inlineStr">
+      <c r="D2177" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
@@ -71755,15 +71755,15 @@
     </row>
     <row r="2179">
       <c r="A2179" s="9" t="n"/>
-      <c r="B2179" t="n">
+      <c r="B2179" s="0" t="n">
         <v>338</v>
       </c>
-      <c r="C2179" t="inlineStr">
+      <c r="C2179" s="0" t="inlineStr">
         <is>
           <t>125, 125</t>
         </is>
       </c>
-      <c r="D2179" t="inlineStr">
+      <c r="D2179" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
@@ -71787,15 +71787,15 @@
     </row>
     <row r="2181">
       <c r="A2181" s="9" t="n"/>
-      <c r="B2181" t="n">
+      <c r="B2181" s="0" t="n">
         <v>338</v>
       </c>
-      <c r="C2181" t="inlineStr">
+      <c r="C2181" s="0" t="inlineStr">
         <is>
           <t>175, 25</t>
         </is>
       </c>
-      <c r="D2181" t="inlineStr">
+      <c r="D2181" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
@@ -71819,15 +71819,15 @@
     </row>
     <row r="2183">
       <c r="A2183" s="9" t="n"/>
-      <c r="B2183" t="n">
+      <c r="B2183" s="0" t="n">
         <v>338</v>
       </c>
-      <c r="C2183" t="inlineStr">
+      <c r="C2183" s="0" t="inlineStr">
         <is>
           <t>175, 125</t>
         </is>
       </c>
-      <c r="D2183" t="inlineStr">
+      <c r="D2183" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
@@ -71888,15 +71888,15 @@
     </row>
     <row r="2188">
       <c r="A2188" s="9" t="n"/>
-      <c r="B2188" t="n">
+      <c r="B2188" s="0" t="n">
         <v>24</v>
       </c>
-      <c r="C2188" t="inlineStr">
+      <c r="C2188" s="0" t="inlineStr">
         <is>
           <t>1, 4</t>
         </is>
       </c>
-      <c r="D2188" t="inlineStr">
+      <c r="D2188" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
@@ -71920,15 +71920,15 @@
     </row>
     <row r="2190">
       <c r="A2190" s="9" t="n"/>
-      <c r="B2190" t="n">
+      <c r="B2190" s="0" t="n">
         <v>28</v>
       </c>
-      <c r="C2190" t="inlineStr">
+      <c r="C2190" s="0" t="inlineStr">
         <is>
           <t>2, 3</t>
         </is>
       </c>
-      <c r="D2190" t="inlineStr">
+      <c r="D2190" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
@@ -72015,15 +72015,15 @@
     </row>
     <row r="2198">
       <c r="A2198" s="9" t="n"/>
-      <c r="B2198" t="n">
+      <c r="B2198" s="0" t="n">
         <v>481</v>
       </c>
-      <c r="C2198" t="inlineStr">
+      <c r="C2198" s="0" t="inlineStr">
         <is>
           <t>9, 6</t>
         </is>
       </c>
-      <c r="D2198" t="inlineStr">
+      <c r="D2198" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
@@ -72039,15 +72039,15 @@
     </row>
     <row r="2200">
       <c r="A2200" s="9" t="n"/>
-      <c r="B2200" t="n">
+      <c r="B2200" s="0" t="n">
         <v>284</v>
       </c>
-      <c r="C2200" t="inlineStr">
+      <c r="C2200" s="0" t="inlineStr">
         <is>
           <t>2, 4</t>
         </is>
       </c>
-      <c r="D2200" t="inlineStr">
+      <c r="D2200" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
@@ -72063,15 +72063,15 @@
     </row>
     <row r="2202">
       <c r="A2202" s="9" t="n"/>
-      <c r="B2202" t="n">
+      <c r="B2202" s="0" t="n">
         <v>281</v>
       </c>
-      <c r="C2202" t="inlineStr">
+      <c r="C2202" s="0" t="inlineStr">
         <is>
           <t>2, 4</t>
         </is>
       </c>
-      <c r="D2202" t="inlineStr">
+      <c r="D2202" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
@@ -72156,15 +72156,15 @@
     </row>
     <row r="2210">
       <c r="A2210" s="9" t="n"/>
-      <c r="B2210" t="n">
+      <c r="B2210" s="0" t="n">
         <v>286</v>
       </c>
-      <c r="C2210" t="inlineStr">
+      <c r="C2210" s="0" t="inlineStr">
         <is>
           <t>14, 11</t>
         </is>
       </c>
-      <c r="D2210" t="inlineStr">
+      <c r="D2210" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
@@ -72204,15 +72204,15 @@
     </row>
     <row r="2214">
       <c r="A2214" s="9" t="n"/>
-      <c r="B2214" t="n">
+      <c r="B2214" s="0" t="n">
         <v>64</v>
       </c>
-      <c r="C2214" t="inlineStr">
+      <c r="C2214" s="0" t="inlineStr">
         <is>
           <t>3, 4</t>
         </is>
       </c>
-      <c r="D2214" t="inlineStr">
+      <c r="D2214" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
@@ -72331,15 +72331,15 @@
     </row>
     <row r="2225">
       <c r="A2225" s="9" t="n"/>
-      <c r="B2225" t="n">
+      <c r="B2225" s="0" t="n">
         <v>271</v>
       </c>
-      <c r="C2225" t="inlineStr">
+      <c r="C2225" s="0" t="inlineStr">
         <is>
           <t>6, 8</t>
         </is>
       </c>
-      <c r="D2225" t="inlineStr">
+      <c r="D2225" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
@@ -72355,15 +72355,15 @@
     </row>
     <row r="2227">
       <c r="A2227" s="9" t="n"/>
-      <c r="B2227" t="n">
+      <c r="B2227" s="0" t="n">
         <v>110</v>
       </c>
-      <c r="C2227" t="inlineStr">
+      <c r="C2227" s="0" t="inlineStr">
         <is>
           <t>5, 10</t>
         </is>
       </c>
-      <c r="D2227" t="inlineStr">
+      <c r="D2227" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
@@ -72379,15 +72379,15 @@
     </row>
     <row r="2229">
       <c r="A2229" s="9" t="n"/>
-      <c r="B2229" t="n">
+      <c r="B2229" s="0" t="n">
         <v>368</v>
       </c>
-      <c r="C2229" t="inlineStr">
+      <c r="C2229" s="0" t="inlineStr">
         <is>
           <t>10, 8</t>
         </is>
       </c>
-      <c r="D2229" t="inlineStr">
+      <c r="D2229" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
@@ -72403,15 +72403,15 @@
     </row>
     <row r="2231">
       <c r="A2231" s="9" t="n"/>
-      <c r="B2231" t="n">
+      <c r="B2231" s="0" t="n">
         <v>369</v>
       </c>
-      <c r="C2231" t="inlineStr">
+      <c r="C2231" s="0" t="inlineStr">
         <is>
           <t>45, 2</t>
         </is>
       </c>
-      <c r="D2231" t="inlineStr">
+      <c r="D2231" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
@@ -72427,15 +72427,15 @@
     </row>
     <row r="2233">
       <c r="A2233" s="9" t="n"/>
-      <c r="B2233" t="n">
+      <c r="B2233" s="0" t="n">
         <v>371</v>
       </c>
-      <c r="C2233" t="inlineStr">
+      <c r="C2233" s="0" t="inlineStr">
         <is>
           <t>6, 3</t>
         </is>
       </c>
-      <c r="D2233" t="inlineStr">
+      <c r="D2233" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
@@ -72480,15 +72480,15 @@
     </row>
     <row r="2237">
       <c r="A2237" s="9" t="n"/>
-      <c r="B2237" t="n">
+      <c r="B2237" s="0" t="n">
         <v>395</v>
       </c>
-      <c r="C2237" t="inlineStr">
+      <c r="C2237" s="0" t="inlineStr">
         <is>
           <t>83, 12</t>
         </is>
       </c>
-      <c r="D2237" t="inlineStr">
+      <c r="D2237" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
@@ -72512,15 +72512,15 @@
     </row>
     <row r="2239">
       <c r="A2239" s="9" t="n"/>
-      <c r="B2239" t="n">
+      <c r="B2239" s="0" t="n">
         <v>397</v>
       </c>
-      <c r="C2239" t="inlineStr">
+      <c r="C2239" s="0" t="inlineStr">
         <is>
           <t>42, 15</t>
         </is>
       </c>
-      <c r="D2239" t="inlineStr">
+      <c r="D2239" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
@@ -72536,15 +72536,15 @@
     </row>
     <row r="2241">
       <c r="A2241" s="9" t="n"/>
-      <c r="B2241" t="n">
+      <c r="B2241" s="0" t="n">
         <v>398</v>
       </c>
-      <c r="C2241" t="inlineStr">
+      <c r="C2241" s="0" t="inlineStr">
         <is>
           <t>24, 52</t>
         </is>
       </c>
-      <c r="D2241" t="inlineStr">
+      <c r="D2241" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
@@ -72568,15 +72568,15 @@
     </row>
     <row r="2243">
       <c r="A2243" s="9" t="n"/>
-      <c r="B2243" t="n">
+      <c r="B2243" s="0" t="n">
         <v>400</v>
       </c>
-      <c r="C2243" t="inlineStr">
+      <c r="C2243" s="0" t="inlineStr">
         <is>
           <t>9, 61</t>
         </is>
       </c>
-      <c r="D2243" t="inlineStr">
+      <c r="D2243" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
@@ -72608,15 +72608,15 @@
     </row>
     <row r="2246">
       <c r="A2246" s="9" t="n"/>
-      <c r="B2246" t="n">
+      <c r="B2246" s="0" t="n">
         <v>405</v>
       </c>
-      <c r="C2246" t="inlineStr">
+      <c r="C2246" s="0" t="inlineStr">
         <is>
           <t>35, 5</t>
         </is>
       </c>
-      <c r="D2246" t="inlineStr">
+      <c r="D2246" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
@@ -72861,365 +72861,365 @@
       </c>
     </row>
     <row r="2269">
-      <c r="A2269" t="n">
+      <c r="A2269" s="0" t="n">
         <v>1912</v>
       </c>
     </row>
     <row r="2270">
-      <c r="B2270" t="n">
+      <c r="B2270" s="0" t="n">
         <v>147</v>
       </c>
-      <c r="C2270" t="inlineStr">
+      <c r="C2270" s="0" t="inlineStr">
         <is>
           <t>9, 7</t>
         </is>
       </c>
-      <c r="D2270" t="inlineStr">
+      <c r="D2270" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
       </c>
     </row>
     <row r="2271">
-      <c r="A2271" t="n">
+      <c r="A2271" s="0" t="n">
         <v>1696</v>
       </c>
     </row>
     <row r="2272">
-      <c r="B2272" t="n">
+      <c r="B2272" s="0" t="n">
         <v>112</v>
       </c>
-      <c r="C2272" t="inlineStr">
+      <c r="C2272" s="0" t="inlineStr">
         <is>
           <t>10, 9</t>
         </is>
       </c>
-      <c r="D2272" t="inlineStr">
+      <c r="D2272" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
       </c>
     </row>
     <row r="2273">
-      <c r="A2273" t="n">
+      <c r="A2273" s="0" t="n">
         <v>1652</v>
       </c>
     </row>
     <row r="2274">
-      <c r="B2274" t="n">
+      <c r="B2274" s="0" t="n">
         <v>129</v>
       </c>
-      <c r="C2274" t="inlineStr">
+      <c r="C2274" s="0" t="inlineStr">
         <is>
           <t>10, 7</t>
         </is>
       </c>
-      <c r="D2274" t="inlineStr">
+      <c r="D2274" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
       </c>
     </row>
     <row r="2275">
-      <c r="B2275" t="n">
+      <c r="B2275" s="0" t="n">
         <v>132</v>
       </c>
-      <c r="C2275" t="inlineStr">
+      <c r="C2275" s="0" t="inlineStr">
         <is>
           <t>8, 7</t>
         </is>
       </c>
-      <c r="D2275" t="inlineStr">
+      <c r="D2275" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
       </c>
     </row>
     <row r="2276">
-      <c r="A2276" t="n">
+      <c r="A2276" s="0" t="n">
         <v>1653</v>
       </c>
     </row>
     <row r="2277">
-      <c r="B2277" t="n">
+      <c r="B2277" s="0" t="n">
         <v>130</v>
       </c>
-      <c r="C2277" t="inlineStr">
+      <c r="C2277" s="0" t="inlineStr">
         <is>
           <t>7, 7</t>
         </is>
       </c>
-      <c r="D2277" t="inlineStr">
+      <c r="D2277" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
       </c>
     </row>
     <row r="2278">
-      <c r="A2278" t="n">
+      <c r="A2278" s="0" t="n">
         <v>1685</v>
       </c>
     </row>
     <row r="2279">
-      <c r="B2279" t="n">
+      <c r="B2279" s="0" t="n">
         <v>272</v>
       </c>
-      <c r="C2279" t="inlineStr">
+      <c r="C2279" s="0" t="inlineStr">
         <is>
           <t>8, 6</t>
         </is>
       </c>
-      <c r="D2279" t="inlineStr">
+      <c r="D2279" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
       </c>
     </row>
     <row r="2280">
-      <c r="A2280" t="n">
+      <c r="A2280" s="0" t="n">
         <v>1674</v>
       </c>
     </row>
     <row r="2281">
-      <c r="B2281" t="n">
+      <c r="B2281" s="0" t="n">
         <v>131</v>
       </c>
-      <c r="C2281" t="inlineStr">
+      <c r="C2281" s="0" t="inlineStr">
         <is>
           <t>10, 7</t>
         </is>
       </c>
-      <c r="D2281" t="inlineStr">
+      <c r="D2281" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
       </c>
     </row>
     <row r="2282">
-      <c r="A2282" t="n">
+      <c r="A2282" s="0" t="n">
         <v>1702</v>
       </c>
     </row>
     <row r="2283">
-      <c r="B2283" t="n">
+      <c r="B2283" s="0" t="n">
         <v>129</v>
       </c>
-      <c r="C2283" t="inlineStr">
+      <c r="C2283" s="0" t="inlineStr">
         <is>
           <t>10, 7</t>
         </is>
       </c>
-      <c r="D2283" t="inlineStr">
+      <c r="D2283" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
       </c>
     </row>
     <row r="2284">
-      <c r="B2284" t="n">
+      <c r="B2284" s="0" t="n">
         <v>132</v>
       </c>
-      <c r="C2284" t="inlineStr">
+      <c r="C2284" s="0" t="inlineStr">
         <is>
           <t>8, 7</t>
         </is>
       </c>
-      <c r="D2284" t="inlineStr">
+      <c r="D2284" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
       </c>
     </row>
     <row r="2285">
-      <c r="A2285" t="n">
+      <c r="A2285" s="0" t="n">
         <v>1703</v>
       </c>
     </row>
     <row r="2286">
-      <c r="B2286" t="n">
+      <c r="B2286" s="0" t="n">
         <v>130</v>
       </c>
-      <c r="C2286" t="inlineStr">
+      <c r="C2286" s="0" t="inlineStr">
         <is>
           <t>7, 7</t>
         </is>
       </c>
-      <c r="D2286" t="inlineStr">
+      <c r="D2286" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
       </c>
     </row>
     <row r="2287">
-      <c r="A2287" t="n">
+      <c r="A2287" s="0" t="n">
         <v>1725</v>
       </c>
     </row>
     <row r="2288">
-      <c r="B2288" t="n">
+      <c r="B2288" s="0" t="n">
         <v>272</v>
       </c>
-      <c r="C2288" t="inlineStr">
+      <c r="C2288" s="0" t="inlineStr">
         <is>
           <t>8, 6</t>
         </is>
       </c>
-      <c r="D2288" t="inlineStr">
+      <c r="D2288" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
       </c>
     </row>
     <row r="2289">
-      <c r="A2289" t="n">
+      <c r="A2289" s="0" t="n">
         <v>1724</v>
       </c>
     </row>
     <row r="2290">
-      <c r="B2290" t="n">
+      <c r="B2290" s="0" t="n">
         <v>131</v>
       </c>
-      <c r="C2290" t="inlineStr">
+      <c r="C2290" s="0" t="inlineStr">
         <is>
           <t>10, 7</t>
         </is>
       </c>
-      <c r="D2290" t="inlineStr">
+      <c r="D2290" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
       </c>
     </row>
     <row r="2291">
-      <c r="A2291" t="n">
+      <c r="A2291" s="0" t="n">
         <v>1998</v>
       </c>
     </row>
     <row r="2292">
-      <c r="B2292" t="n">
+      <c r="B2292" s="0" t="n">
         <v>625</v>
       </c>
-      <c r="C2292" t="inlineStr">
+      <c r="C2292" s="0" t="inlineStr">
         <is>
           <t>14, 19</t>
         </is>
       </c>
-      <c r="D2292" t="inlineStr">
+      <c r="D2292" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
       </c>
     </row>
     <row r="2293">
-      <c r="A2293" t="n">
+      <c r="A2293" s="0" t="n">
         <v>2001</v>
       </c>
     </row>
     <row r="2294">
-      <c r="B2294" t="n">
+      <c r="B2294" s="0" t="n">
         <v>625</v>
       </c>
-      <c r="C2294" t="inlineStr">
+      <c r="C2294" s="0" t="inlineStr">
         <is>
           <t>14, 19</t>
         </is>
       </c>
-      <c r="D2294" t="inlineStr">
+      <c r="D2294" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
       </c>
     </row>
     <row r="2295">
-      <c r="A2295" t="n">
+      <c r="A2295" s="0" t="n">
         <v>2042</v>
       </c>
     </row>
     <row r="2296">
-      <c r="B2296" t="n">
+      <c r="B2296" s="0" t="n">
         <v>625</v>
       </c>
-      <c r="C2296" t="inlineStr">
+      <c r="C2296" s="0" t="inlineStr">
         <is>
           <t>14, 19</t>
         </is>
       </c>
-      <c r="D2296" t="inlineStr">
+      <c r="D2296" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
       </c>
     </row>
     <row r="2297">
-      <c r="A2297" t="n">
+      <c r="A2297" s="0" t="n">
         <v>2004</v>
       </c>
     </row>
     <row r="2298">
-      <c r="B2298" t="n">
+      <c r="B2298" s="0" t="n">
         <v>625</v>
       </c>
-      <c r="C2298" t="inlineStr">
+      <c r="C2298" s="0" t="inlineStr">
         <is>
           <t>14, 19</t>
         </is>
       </c>
-      <c r="D2298" t="inlineStr">
+      <c r="D2298" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
       </c>
     </row>
     <row r="2299">
-      <c r="A2299" t="n">
+      <c r="A2299" s="0" t="n">
         <v>46011</v>
       </c>
     </row>
     <row r="2300">
-      <c r="B2300" t="n">
+      <c r="B2300" s="0" t="n">
         <v>608</v>
       </c>
-      <c r="C2300" t="inlineStr">
+      <c r="C2300" s="0" t="inlineStr">
         <is>
           <t>15, 8</t>
         </is>
       </c>
-      <c r="D2300" t="inlineStr">
+      <c r="D2300" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
       </c>
     </row>
     <row r="2301">
-      <c r="B2301" t="n">
+      <c r="B2301" s="0" t="n">
         <v>609</v>
       </c>
-      <c r="C2301" t="inlineStr">
+      <c r="C2301" s="0" t="inlineStr">
         <is>
           <t>14, 14</t>
         </is>
       </c>
-      <c r="D2301" t="inlineStr">
+      <c r="D2301" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
       </c>
     </row>
     <row r="2302">
-      <c r="A2302" t="n">
+      <c r="A2302" s="0" t="n">
         <v>6517</v>
       </c>
     </row>
     <row r="2303">
-      <c r="B2303" t="n">
+      <c r="B2303" s="0" t="n">
         <v>64</v>
       </c>
-      <c r="C2303" t="inlineStr">
+      <c r="C2303" s="0" t="inlineStr">
         <is>
           <t>3, 4</t>
         </is>
       </c>
-      <c r="D2303" t="inlineStr">
+      <c r="D2303" s="0" t="inlineStr">
         <is>
           <t>BOTTOM</t>
         </is>
@@ -73237,7 +73237,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="9" customWidth="1" style="2" min="1" max="5"/>
@@ -73281,24 +73281,455 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="B4" s="4" t="n"/>
+      <c r="A4" t="n">
+        <v>34</v>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="n"/>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>혼잣말1</t>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>여기는 초보자사냥터입니다.초보자에게 적합한 던전으로,1 레벨부터 10 레벨까지 사냥하기에 좋습니다.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="n"/>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>혼잣말2</t>
+      <c r="A6" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>여기는 쥐굴입니다. 초보자에게 적합한 던전으로,5 레벨부터 10 레벨까지 사냥하기에 좋습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>여기는 사슴굴입니다. 10 레벨부터 25 레벨까지 사냥하기에좋습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>여기는 돼지굴입니다. 30 레벨부터 45 레벨까지 사냥하기에좋습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>여기는 곰굴입니다. 20 레벨부터 40 레벨까지 사냥하기에 좋습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>여기는 여우굴입니다. 30 레벨부터 45 레벨까지 사냥하기에 좋습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>여기는 인형굴입니다. 60 레벨부터 80 레벨까지 사냥하기에좋습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>여기는 해골굴입니다. 60 레벨부터 90 레벨까지 사냥하기에좋습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>여기는 유령굴입니다. 60 레벨부터 90 레벨까지 사냥하기에좋습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>여기는 흑해골굴입니다. 65 레벨부터 90 레벨까지 사냥하기에좋습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>여기는 흑령굴입니다. 65 레벨부터 90 레벨까지 사냥하기에좋습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>여기는 사마귀굴입니다. 55 레벨부터 70 레벨까지 사냥하기에좋습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>여기는 전갈굴입니다. 55 레벨부터 70 레벨까지 사냥하기에좋습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>여기는 백륜동입니다. 80 레벨부터 99 레벨까지 사냥하기에좋습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>여기는 물망동입니다. 80 레벨부터 99 레벨까지 사냥하기에좋습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>여기는 흉가입니다. 95 레벨부터 99 레벨 이상 고레벨이 사냥하기에 좋습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>여기는 자호굴입니다. 40 레벨부터 60 레벨까지 사냥하기에좋습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>여기는 비밀세작의 집입니다.85 레벨부터 99 레벨 이상 고레벨이 사냥하기에 좋습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>땅에 떨어져서 흙이 묻은 얼음을 씻어드립니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>깨끗한 얼음이 있어야 화채를 만드실 수 있답니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>말하는 방법을 모르신다구요? 그러면 저를 클릭해 보세요.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>단계를 모두 완료하시면 경험치를 드리고 있어요.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>홈페이지가 어딘지 궁금하다면...? F2키를...</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>저는 수련방법을 알려드리는 사냥도우미라고 합니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>저 넓은 세계 어딘가에는 많은 사람들이 있다고 하던데...</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>제가 드린 퀘스트를 완료하시면 약간의 경험치를 드립니다...</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>바람의나라에 대해 잘 모르신다구요? 그럼 저 똘똘이 도우미가 알려드리겠습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>열심히 공부한 학생에게는 약간의 상이 있을지도 없을지도?</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>언제나 탐구하는 자세를 가지고 정진하시길 바랍니다...</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>안녕하세요? 저를 클릭 해 보세요.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>안녕하세요?</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>세상에는 너무나 많은 아이템이 존재합니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>적절한 아이템을 쓰는 것이 곧 고수가 되는 길...</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>말하기는 [ENTER]키를 누르시면 가능합니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>직업 선생님들은 도토리와 토끼고기를 좋아하시는 것 같던데...</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>님이 하고싶은 직업은 남들도 하고싶어요. 그러니 도사를 하는게 어떠세요?</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>도사가 없는게 아니고,님이 도사를 안한거에요.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>상대방의 체력이 너무 높다고...? 그러면 방어력을 낮추면 되지...</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>방어력을 낮추는 마법은 저주와 혼마술이 있지...</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>방어력무시라는 특수한 각인이 있는데,이건 비밀이니 조용히 해야돼요...</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>부여성에 오신걸 환영합니다~</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>반갑습니다. 제 이름은 률이라고 합니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>F2를 눌러 메일주소를 등록해 주시기 바랍니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>저 넓은 세계에는 무엇이 있을까요...</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: swap Gogyundo ticket NPC spawns
- Place the Buyeo ticket NPC on the Buyeo pier
- Place the Goguryeo ticket NPC on the Goguryeo pier
</commit_message>
<xml_diff>
--- a/resources/table/npc.xlsx
+++ b/resources/table/npc.xlsx
@@ -63335,7 +63335,7 @@
       <c r="A1512" s="3" t="n"/>
       <c r="B1512" s="4" t="inlineStr">
         <is>
-          <t>199</t>
+          <t>198</t>
         </is>
       </c>
       <c r="C1512" s="4" t="inlineStr">
@@ -63391,7 +63391,7 @@
       <c r="A1516" s="4" t="n"/>
       <c r="B1516" s="3" t="inlineStr">
         <is>
-          <t>198</t>
+          <t>199</t>
         </is>
       </c>
       <c r="C1516" s="3" t="inlineStr">

</xml_diff>